<commit_message>
Release v2.0.0 with expanded research and comparison tools
</commit_message>
<xml_diff>
--- a/시장조사.xlsx
+++ b/시장조사.xlsx
@@ -1407,7 +1407,35 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">(StatCounter 2026-09)</t>
+      <t xml:space="preserve">(StatCounter 2026-09) · </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">게임전략 파일 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4-7</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">에 참조용 복사본 있음</t>
     </r>
   </si>
   <si>
@@ -5443,16 +5471,50 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">광고 채널</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(3-2)·</t>
+      <t xml:space="preserve">광고 채널 분석</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(3-2)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">의 채널별 게임 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">CPI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 확인 불가</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
     </r>
     <r>
       <rPr>
@@ -5469,7 +5531,160 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">(3-3)·</t>
+      <t xml:space="preserve">(3-3)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">은 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">AdWhispr </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">분류</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">게임당 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">25</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개 표본</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) + </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">영상 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">30</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개 처음 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">초 분석자 판독</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">화면 캡처 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2~3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">장 기준</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">). </t>
     </r>
     <r>
       <rPr>
@@ -5494,7 +5709,7 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">은 다음 창에서 진행</t>
+      <t xml:space="preserve">은 전부 분석자 제안</t>
     </r>
     <r>
       <rPr>
@@ -20622,38 +20837,101 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">(1-4 </t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="11"/>
-        <color rgb="FF595959"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">세부 장르 시트에는 없음 — </t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="11"/>
-        <color rgb="FF595959"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1-4</t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="11"/>
-        <color rgb="FF595959"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">는 </t>
+      <t xml:space="preserve">(6</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="11"/>
+        <color rgb="FF595959"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">단계</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="11"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">-3</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="11"/>
+        <color rgb="FF595959"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">에서 </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="11"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">'1-4 </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="11"/>
+        <color rgb="FF595959"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">세부 장르</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="11"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">' </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="11"/>
+        <color rgb="FF595959"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">맨 아래 별도 표에 추가함 — </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="11"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1-4 </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="11"/>
+        <color rgb="FF595959"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">위쪽 표는 </t>
     </r>
     <r>
       <rPr>
@@ -32522,11 +32800,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="27132666"/>
-        <c:axId val="63404222"/>
+        <c:axId val="81340221"/>
+        <c:axId val="6678366"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="27132666"/>
+        <c:axId val="81340221"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -32558,7 +32836,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="63404222"/>
+        <c:crossAx val="6678366"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -32566,7 +32844,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="63404222"/>
+        <c:axId val="6678366"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -32642,7 +32920,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="27132666"/>
+        <c:crossAx val="81340221"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -33893,11 +34171,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="22527595"/>
-        <c:axId val="91440010"/>
+        <c:axId val="13348130"/>
+        <c:axId val="19480753"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="22527595"/>
+        <c:axId val="13348130"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -33929,7 +34207,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="91440010"/>
+        <c:crossAx val="19480753"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -33937,7 +34215,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="91440010"/>
+        <c:axId val="19480753"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -34013,7 +34291,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="22527595"/>
+        <c:crossAx val="13348130"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -49674,7 +49952,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="48.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
         <v>104</v>
       </c>

</xml_diff>